<commit_message>
Carry group strategy notes into each intake file
Copies the bottom-of-sheet details from the July 2026 master (General
Strategy, Initiatives, List # tables, and Blitz calendars for
FE/BE/PCO/Auto) into a formatted panel to the right of the schedule
table in each group's pre-filled intake file.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DBbqxUN9AD2FdtJjEWSJGT
</commit_message>
<xml_diff>
--- a/call-delivery/intake/2026-07/Auto.xlsx
+++ b/call-delivery/intake/2026-07/Auto.xlsx
@@ -17,11 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="mm/dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +55,24 @@
     </font>
     <font>
       <color rgb="006B7280"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E5AAC"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2A44"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -105,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -122,7 +141,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -131,7 +150,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -144,6 +163,38 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -527,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I186"/>
+  <dimension ref="B2:N186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -539,12 +590,21 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="24" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
           <t>CALL DELIVERY  —  Outbound Dialing Schedule (Intake)</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>GROUP STRATEGY &amp; NOTES  (carried over from July 2026 master)</t>
         </is>
       </c>
     </row>
@@ -555,6 +615,13 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>General Strategy</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -576,6 +643,11 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K5" s="16" t="inlineStr">
+        <is>
+          <t>M-F (2) Full Passes</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="B6" s="3" t="inlineStr">
@@ -593,8 +665,27 @@
           <t>Submitted Date:</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="17" t="n">
         <v>46220</v>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>Initiatives</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>No Slow Volume for the 1st (4) days.  Don't schedule dedicated passes until 5th</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>Adding a WFO Only pass in the afternoons</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -638,13 +729,18 @@
           <t>Special Instructions</t>
         </is>
       </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>No passes after 4:00p due to staffing</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="18" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="10" t="n">
@@ -679,7 +775,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="18" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="10" t="n">
@@ -704,13 +800,18 @@
         </is>
       </c>
       <c r="I11" s="12" t="n"/>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>Lists</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="18" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="10" t="n">
@@ -731,13 +832,28 @@
         </is>
       </c>
       <c r="I12" s="12" t="n"/>
+      <c r="K12" s="19" t="inlineStr">
+        <is>
+          <t>List #</t>
+        </is>
+      </c>
+      <c r="L12" s="19" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="M12" s="19" t="inlineStr">
+        <is>
+          <t>List Specific Strategy</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13" s="18" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="10" t="n">
@@ -758,13 +874,26 @@
         </is>
       </c>
       <c r="I13" s="12" t="n"/>
+      <c r="K13" s="20" t="n">
+        <v>26100</v>
+      </c>
+      <c r="L13" s="21" t="inlineStr">
+        <is>
+          <t>AUTODRCCT_1PLUS</t>
+        </is>
+      </c>
+      <c r="M13" s="21" t="inlineStr">
+        <is>
+          <t>All Auto Passes (except dedicated Slow Only)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="18" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="10" t="n">
@@ -785,13 +914,26 @@
         </is>
       </c>
       <c r="I14" s="12" t="n"/>
+      <c r="K14" s="20" t="n">
+        <v>26101</v>
+      </c>
+      <c r="L14" s="21" t="inlineStr">
+        <is>
+          <t>AUTODRCCT_SLOWPAY</t>
+        </is>
+      </c>
+      <c r="M14" s="21" t="inlineStr">
+        <is>
+          <t>All Auto Passes (except dedicated 1Pay)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C15" s="9" t="n">
+      <c r="C15" s="18" t="n">
         <v>46205</v>
       </c>
       <c r="D15" s="10" t="n">
@@ -816,13 +958,26 @@
           <t>Slowpay AM Daily</t>
         </is>
       </c>
+      <c r="K15" s="20" t="n">
+        <v>17101</v>
+      </c>
+      <c r="L15" s="21" t="inlineStr">
+        <is>
+          <t>LSC_AUTO_FE</t>
+        </is>
+      </c>
+      <c r="M15" s="21" t="inlineStr">
+        <is>
+          <t>All Auto Passes (except dedicated Slow Only)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="18" t="n">
         <v>46205</v>
       </c>
       <c r="D16" s="10" t="n">
@@ -849,7 +1004,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="18" t="n">
         <v>46205</v>
       </c>
       <c r="D17" s="10" t="n">
@@ -870,13 +1025,18 @@
         </is>
       </c>
       <c r="I17" s="12" t="n"/>
+      <c r="K17" s="15" t="inlineStr">
+        <is>
+          <t>Blitz Calendar</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="18" t="n">
         <v>46205</v>
       </c>
       <c r="D18" s="10" t="n">
@@ -897,13 +1057,33 @@
         </is>
       </c>
       <c r="I18" s="12" t="n"/>
+      <c r="K18" s="19" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="L18" s="19" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="M18" s="19" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="N18" s="19" t="inlineStr">
+        <is>
+          <t>FE PM</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="18" t="n">
         <v>46205</v>
       </c>
       <c r="D19" s="10" t="n">
@@ -924,13 +1104,27 @@
         </is>
       </c>
       <c r="I19" s="12" t="n"/>
+      <c r="K19" s="22" t="n">
+        <v>46204</v>
+      </c>
+      <c r="L19" s="20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="M19" s="20" t="n"/>
+      <c r="N19" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C20" s="18" t="n">
         <v>46209</v>
       </c>
       <c r="D20" s="10" t="n">
@@ -959,13 +1153,27 @@
           <t>Slowpay AM Daily</t>
         </is>
       </c>
+      <c r="K20" s="22" t="n">
+        <v>46205</v>
+      </c>
+      <c r="L20" s="20" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="M20" s="20" t="n"/>
+      <c r="N20" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C21" s="18" t="n">
         <v>46209</v>
       </c>
       <c r="D21" s="10" t="n">
@@ -990,13 +1198,23 @@
         </is>
       </c>
       <c r="I21" s="12" t="n"/>
+      <c r="K21" s="22" t="n">
+        <v>46206</v>
+      </c>
+      <c r="L21" s="20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="M21" s="20" t="n"/>
+      <c r="N21" s="20" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="18" t="n">
         <v>46209</v>
       </c>
       <c r="D22" s="10" t="n">
@@ -1017,13 +1235,23 @@
         </is>
       </c>
       <c r="I22" s="12" t="n"/>
+      <c r="K22" s="22" t="n">
+        <v>46207</v>
+      </c>
+      <c r="L22" s="20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="M22" s="20" t="n"/>
+      <c r="N22" s="20" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="18" t="n">
         <v>46209</v>
       </c>
       <c r="D23" s="10" t="n">
@@ -1044,13 +1272,23 @@
         </is>
       </c>
       <c r="I23" s="12" t="n"/>
+      <c r="K23" s="22" t="n">
+        <v>46208</v>
+      </c>
+      <c r="L23" s="20" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="M23" s="20" t="n"/>
+      <c r="N23" s="20" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C24" s="9" t="n">
+      <c r="C24" s="18" t="n">
         <v>46209</v>
       </c>
       <c r="D24" s="10" t="n">
@@ -1071,13 +1309,27 @@
         </is>
       </c>
       <c r="I24" s="12" t="n"/>
+      <c r="K24" s="22" t="n">
+        <v>46209</v>
+      </c>
+      <c r="L24" s="20" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="M24" s="20" t="n"/>
+      <c r="N24" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C25" s="9" t="n">
+      <c r="C25" s="18" t="n">
         <v>46210</v>
       </c>
       <c r="D25" s="10" t="n">
@@ -1102,13 +1354,27 @@
           <t>Slowpay AM Daily</t>
         </is>
       </c>
+      <c r="K25" s="22" t="n">
+        <v>46210</v>
+      </c>
+      <c r="L25" s="20" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="M25" s="20" t="n"/>
+      <c r="N25" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C26" s="9" t="n">
+      <c r="C26" s="18" t="n">
         <v>46210</v>
       </c>
       <c r="D26" s="10" t="n">
@@ -1129,13 +1395,27 @@
       </c>
       <c r="H26" s="11" t="n"/>
       <c r="I26" s="12" t="n"/>
+      <c r="K26" s="22" t="n">
+        <v>46211</v>
+      </c>
+      <c r="L26" s="20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="M26" s="20" t="n"/>
+      <c r="N26" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C27" s="9" t="n">
+      <c r="C27" s="18" t="n">
         <v>46210</v>
       </c>
       <c r="D27" s="10" t="n">
@@ -1156,13 +1436,23 @@
         </is>
       </c>
       <c r="I27" s="12" t="n"/>
+      <c r="K27" s="22" t="n">
+        <v>46212</v>
+      </c>
+      <c r="L27" s="20" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="M27" s="20" t="n"/>
+      <c r="N27" s="20" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C28" s="9" t="n">
+      <c r="C28" s="18" t="n">
         <v>46210</v>
       </c>
       <c r="D28" s="10" t="n">
@@ -1183,13 +1473,27 @@
         </is>
       </c>
       <c r="I28" s="12" t="n"/>
+      <c r="K28" s="22" t="n">
+        <v>46213</v>
+      </c>
+      <c r="L28" s="20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="M28" s="20" t="n"/>
+      <c r="N28" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C29" s="9" t="n">
+      <c r="C29" s="18" t="n">
         <v>46210</v>
       </c>
       <c r="D29" s="10" t="n">
@@ -1210,13 +1514,27 @@
         </is>
       </c>
       <c r="I29" s="12" t="n"/>
+      <c r="K29" s="22" t="n">
+        <v>46214</v>
+      </c>
+      <c r="L29" s="20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="M29" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C30" s="9" t="n">
+      <c r="C30" s="18" t="n">
         <v>46211</v>
       </c>
       <c r="D30" s="10" t="n">
@@ -1245,13 +1563,27 @@
           <t>Slowpay AM Daily</t>
         </is>
       </c>
+      <c r="K30" s="22" t="n">
+        <v>46215</v>
+      </c>
+      <c r="L30" s="20" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="M30" s="20" t="n"/>
+      <c r="N30" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C31" s="9" t="n">
+      <c r="C31" s="18" t="n">
         <v>46211</v>
       </c>
       <c r="D31" s="10" t="n">
@@ -1276,13 +1608,27 @@
         </is>
       </c>
       <c r="I31" s="12" t="n"/>
+      <c r="K31" s="22" t="n">
+        <v>46216</v>
+      </c>
+      <c r="L31" s="20" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="M31" s="20" t="n"/>
+      <c r="N31" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C32" s="9" t="n">
+      <c r="C32" s="18" t="n">
         <v>46211</v>
       </c>
       <c r="D32" s="10" t="n">
@@ -1303,13 +1649,23 @@
         </is>
       </c>
       <c r="I32" s="12" t="n"/>
+      <c r="K32" s="22" t="n">
+        <v>46217</v>
+      </c>
+      <c r="L32" s="20" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="M32" s="20" t="n"/>
+      <c r="N32" s="20" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C33" s="9" t="n">
+      <c r="C33" s="18" t="n">
         <v>46211</v>
       </c>
       <c r="D33" s="10" t="n">
@@ -1330,13 +1686,27 @@
         </is>
       </c>
       <c r="I33" s="12" t="n"/>
+      <c r="K33" s="22" t="n">
+        <v>46218</v>
+      </c>
+      <c r="L33" s="20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="M33" s="20" t="n"/>
+      <c r="N33" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C34" s="9" t="n">
+      <c r="C34" s="18" t="n">
         <v>46211</v>
       </c>
       <c r="D34" s="10" t="n">
@@ -1357,13 +1727,23 @@
         </is>
       </c>
       <c r="I34" s="12" t="n"/>
+      <c r="K34" s="22" t="n">
+        <v>46219</v>
+      </c>
+      <c r="L34" s="20" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="M34" s="20" t="n"/>
+      <c r="N34" s="20" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C35" s="9" t="n">
+      <c r="C35" s="18" t="n">
         <v>46212</v>
       </c>
       <c r="D35" s="10" t="n">
@@ -1388,13 +1768,27 @@
           <t>Slowpay AM Daily</t>
         </is>
       </c>
+      <c r="K35" s="22" t="n">
+        <v>46220</v>
+      </c>
+      <c r="L35" s="20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="M35" s="20" t="n"/>
+      <c r="N35" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C36" s="9" t="n">
+      <c r="C36" s="18" t="n">
         <v>46212</v>
       </c>
       <c r="D36" s="10" t="n">
@@ -1415,13 +1809,31 @@
       </c>
       <c r="H36" s="11" t="n"/>
       <c r="I36" s="12" t="n"/>
+      <c r="K36" s="22" t="n">
+        <v>46221</v>
+      </c>
+      <c r="L36" s="20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="M36" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N36" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C37" s="9" t="n">
+      <c r="C37" s="18" t="n">
         <v>46212</v>
       </c>
       <c r="D37" s="10" t="n">
@@ -1442,13 +1854,27 @@
         </is>
       </c>
       <c r="I37" s="12" t="n"/>
+      <c r="K37" s="22" t="n">
+        <v>46222</v>
+      </c>
+      <c r="L37" s="20" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="M37" s="20" t="n"/>
+      <c r="N37" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C38" s="9" t="n">
+      <c r="C38" s="18" t="n">
         <v>46212</v>
       </c>
       <c r="D38" s="10" t="n">
@@ -1469,13 +1895,27 @@
       </c>
       <c r="H38" s="11" t="n"/>
       <c r="I38" s="12" t="n"/>
+      <c r="K38" s="22" t="n">
+        <v>46223</v>
+      </c>
+      <c r="L38" s="20" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="M38" s="20" t="n"/>
+      <c r="N38" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C39" s="9" t="n">
+      <c r="C39" s="18" t="n">
         <v>46212</v>
       </c>
       <c r="D39" s="10" t="n">
@@ -1496,13 +1936,23 @@
         </is>
       </c>
       <c r="I39" s="12" t="n"/>
+      <c r="K39" s="22" t="n">
+        <v>46224</v>
+      </c>
+      <c r="L39" s="20" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="M39" s="20" t="n"/>
+      <c r="N39" s="20" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C40" s="9" t="n">
+      <c r="C40" s="18" t="n">
         <v>46213</v>
       </c>
       <c r="D40" s="10" t="n">
@@ -1531,13 +1981,27 @@
           <t>Slowpay AM Daily</t>
         </is>
       </c>
+      <c r="K40" s="22" t="n">
+        <v>46225</v>
+      </c>
+      <c r="L40" s="20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="M40" s="20" t="n"/>
+      <c r="N40" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C41" s="9" t="n">
+      <c r="C41" s="18" t="n">
         <v>46213</v>
       </c>
       <c r="D41" s="10" t="n">
@@ -1562,13 +2026,23 @@
         </is>
       </c>
       <c r="I41" s="12" t="n"/>
+      <c r="K41" s="22" t="n">
+        <v>46226</v>
+      </c>
+      <c r="L41" s="20" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="M41" s="20" t="n"/>
+      <c r="N41" s="20" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C42" s="9" t="n">
+      <c r="C42" s="18" t="n">
         <v>46213</v>
       </c>
       <c r="D42" s="10" t="n">
@@ -1589,13 +2063,27 @@
         </is>
       </c>
       <c r="I42" s="12" t="n"/>
+      <c r="K42" s="22" t="n">
+        <v>46227</v>
+      </c>
+      <c r="L42" s="20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="M42" s="20" t="n"/>
+      <c r="N42" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C43" s="9" t="n">
+      <c r="C43" s="18" t="n">
         <v>46213</v>
       </c>
       <c r="D43" s="10" t="n">
@@ -1616,13 +2104,31 @@
         </is>
       </c>
       <c r="I43" s="12" t="n"/>
+      <c r="K43" s="22" t="n">
+        <v>46228</v>
+      </c>
+      <c r="L43" s="20" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="M43" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="N43" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C44" s="9" t="n">
+      <c r="C44" s="18" t="n">
         <v>46213</v>
       </c>
       <c r="D44" s="10" t="n">
@@ -1643,13 +2149,27 @@
         </is>
       </c>
       <c r="I44" s="12" t="n"/>
+      <c r="K44" s="22" t="n">
+        <v>46229</v>
+      </c>
+      <c r="L44" s="20" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="M44" s="20" t="n"/>
+      <c r="N44" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C45" s="9" t="n">
+      <c r="C45" s="18" t="n">
         <v>46214</v>
       </c>
       <c r="D45" s="10" t="n">
@@ -1670,13 +2190,27 @@
         </is>
       </c>
       <c r="I45" s="12" t="n"/>
+      <c r="K45" s="22" t="n">
+        <v>46230</v>
+      </c>
+      <c r="L45" s="20" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="M45" s="20" t="n"/>
+      <c r="N45" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C46" s="9" t="n">
+      <c r="C46" s="18" t="n">
         <v>46215</v>
       </c>
       <c r="D46" s="10" t="n">
@@ -1697,13 +2231,27 @@
         </is>
       </c>
       <c r="I46" s="12" t="n"/>
+      <c r="K46" s="22" t="n">
+        <v>46231</v>
+      </c>
+      <c r="L46" s="20" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="M46" s="20" t="n"/>
+      <c r="N46" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C47" s="9" t="n">
+      <c r="C47" s="18" t="n">
         <v>46216</v>
       </c>
       <c r="D47" s="10" t="n">
@@ -1732,13 +2280,27 @@
           <t>Slowpay AM Daily</t>
         </is>
       </c>
+      <c r="K47" s="22" t="n">
+        <v>46232</v>
+      </c>
+      <c r="L47" s="20" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="M47" s="20" t="n"/>
+      <c r="N47" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C48" s="9" t="n">
+      <c r="C48" s="18" t="n">
         <v>46216</v>
       </c>
       <c r="D48" s="10" t="n">
@@ -1763,13 +2325,27 @@
         </is>
       </c>
       <c r="I48" s="12" t="n"/>
+      <c r="K48" s="22" t="n">
+        <v>46233</v>
+      </c>
+      <c r="L48" s="20" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="M48" s="20" t="n"/>
+      <c r="N48" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C49" s="9" t="n">
+      <c r="C49" s="18" t="n">
         <v>46216</v>
       </c>
       <c r="D49" s="10" t="n">
@@ -1790,13 +2366,27 @@
         </is>
       </c>
       <c r="I49" s="12" t="n"/>
+      <c r="K49" s="22" t="n">
+        <v>46234</v>
+      </c>
+      <c r="L49" s="20" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="M49" s="20" t="n"/>
+      <c r="N49" s="23" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C50" s="9" t="n">
+      <c r="C50" s="18" t="n">
         <v>46216</v>
       </c>
       <c r="D50" s="10" t="n">
@@ -1817,13 +2407,21 @@
         </is>
       </c>
       <c r="I50" s="12" t="n"/>
+      <c r="L50" s="24" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="M50" s="25" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C51" s="9" t="n">
+      <c r="C51" s="18" t="n">
         <v>46216</v>
       </c>
       <c r="D51" s="10" t="n">
@@ -1850,7 +2448,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C52" s="9" t="n">
+      <c r="C52" s="18" t="n">
         <v>46217</v>
       </c>
       <c r="D52" s="10" t="n">
@@ -1881,7 +2479,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C53" s="9" t="n">
+      <c r="C53" s="18" t="n">
         <v>46217</v>
       </c>
       <c r="D53" s="10" t="n">
@@ -1908,7 +2506,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C54" s="9" t="n">
+      <c r="C54" s="18" t="n">
         <v>46217</v>
       </c>
       <c r="D54" s="10" t="n">
@@ -1935,7 +2533,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C55" s="9" t="n">
+      <c r="C55" s="18" t="n">
         <v>46217</v>
       </c>
       <c r="D55" s="10" t="n">
@@ -1962,7 +2560,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C56" s="9" t="n">
+      <c r="C56" s="18" t="n">
         <v>46217</v>
       </c>
       <c r="D56" s="10" t="n">
@@ -1989,7 +2587,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C57" s="9" t="n">
+      <c r="C57" s="18" t="n">
         <v>46217</v>
       </c>
       <c r="D57" s="10" t="n">
@@ -2016,7 +2614,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C58" s="9" t="n">
+      <c r="C58" s="18" t="n">
         <v>46218</v>
       </c>
       <c r="D58" s="10" t="n">
@@ -2051,7 +2649,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C59" s="9" t="n">
+      <c r="C59" s="18" t="n">
         <v>46218</v>
       </c>
       <c r="D59" s="10" t="n">
@@ -2082,7 +2680,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C60" s="9" t="n">
+      <c r="C60" s="18" t="n">
         <v>46218</v>
       </c>
       <c r="D60" s="10" t="n">
@@ -2109,7 +2707,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C61" s="9" t="n">
+      <c r="C61" s="18" t="n">
         <v>46218</v>
       </c>
       <c r="D61" s="10" t="n">
@@ -2136,7 +2734,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C62" s="9" t="n">
+      <c r="C62" s="18" t="n">
         <v>46218</v>
       </c>
       <c r="D62" s="10" t="n">
@@ -2163,7 +2761,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C63" s="9" t="n">
+      <c r="C63" s="18" t="n">
         <v>46219</v>
       </c>
       <c r="D63" s="10" t="n">
@@ -2194,7 +2792,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C64" s="9" t="n">
+      <c r="C64" s="18" t="n">
         <v>46219</v>
       </c>
       <c r="D64" s="10" t="n">
@@ -2221,7 +2819,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C65" s="9" t="n">
+      <c r="C65" s="18" t="n">
         <v>46219</v>
       </c>
       <c r="D65" s="10" t="n">
@@ -2248,7 +2846,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C66" s="9" t="n">
+      <c r="C66" s="18" t="n">
         <v>46219</v>
       </c>
       <c r="D66" s="10" t="n">
@@ -2275,7 +2873,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C67" s="9" t="n">
+      <c r="C67" s="18" t="n">
         <v>46219</v>
       </c>
       <c r="D67" s="10" t="n">
@@ -2302,7 +2900,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C68" s="9" t="n">
+      <c r="C68" s="18" t="n">
         <v>46219</v>
       </c>
       <c r="D68" s="10" t="n">
@@ -2329,7 +2927,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C69" s="9" t="n">
+      <c r="C69" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D69" s="10" t="n">
@@ -2364,7 +2962,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C70" s="9" t="n">
+      <c r="C70" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D70" s="10" t="n">
@@ -2395,7 +2993,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C71" s="9" t="n">
+      <c r="C71" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D71" s="10" t="n">
@@ -2422,7 +3020,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C72" s="9" t="n">
+      <c r="C72" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D72" s="10" t="n">
@@ -2449,7 +3047,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C73" s="9" t="n">
+      <c r="C73" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D73" s="10" t="n">
@@ -2476,7 +3074,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C74" s="9" t="n">
+      <c r="C74" s="18" t="n">
         <v>46221</v>
       </c>
       <c r="D74" s="10" t="n">
@@ -2503,7 +3101,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C75" s="9" t="n">
+      <c r="C75" s="18" t="n">
         <v>46221</v>
       </c>
       <c r="D75" s="10" t="n">
@@ -2530,7 +3128,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C76" s="9" t="n">
+      <c r="C76" s="18" t="n">
         <v>46222</v>
       </c>
       <c r="D76" s="10" t="n">
@@ -2557,7 +3155,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C77" s="9" t="n">
+      <c r="C77" s="18" t="n">
         <v>46223</v>
       </c>
       <c r="D77" s="10" t="n">
@@ -2592,7 +3190,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C78" s="9" t="n">
+      <c r="C78" s="18" t="n">
         <v>46223</v>
       </c>
       <c r="D78" s="10" t="n">
@@ -2623,7 +3221,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C79" s="9" t="n">
+      <c r="C79" s="18" t="n">
         <v>46223</v>
       </c>
       <c r="D79" s="10" t="n">
@@ -2650,7 +3248,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C80" s="9" t="n">
+      <c r="C80" s="18" t="n">
         <v>46223</v>
       </c>
       <c r="D80" s="10" t="n">
@@ -2677,7 +3275,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C81" s="9" t="n">
+      <c r="C81" s="18" t="n">
         <v>46223</v>
       </c>
       <c r="D81" s="10" t="n">
@@ -2704,7 +3302,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C82" s="9" t="n">
+      <c r="C82" s="18" t="n">
         <v>46224</v>
       </c>
       <c r="D82" s="10" t="n">
@@ -2735,7 +3333,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C83" s="9" t="n">
+      <c r="C83" s="18" t="n">
         <v>46224</v>
       </c>
       <c r="D83" s="10" t="n">
@@ -2762,7 +3360,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C84" s="9" t="n">
+      <c r="C84" s="18" t="n">
         <v>46224</v>
       </c>
       <c r="D84" s="10" t="n">
@@ -2789,7 +3387,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C85" s="9" t="n">
+      <c r="C85" s="18" t="n">
         <v>46224</v>
       </c>
       <c r="D85" s="10" t="n">
@@ -2816,7 +3414,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C86" s="9" t="n">
+      <c r="C86" s="18" t="n">
         <v>46224</v>
       </c>
       <c r="D86" s="10" t="n">
@@ -2843,7 +3441,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C87" s="9" t="n">
+      <c r="C87" s="18" t="n">
         <v>46224</v>
       </c>
       <c r="D87" s="10" t="n">
@@ -2870,7 +3468,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C88" s="9" t="n">
+      <c r="C88" s="18" t="n">
         <v>46225</v>
       </c>
       <c r="D88" s="10" t="n">
@@ -2905,7 +3503,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C89" s="9" t="n">
+      <c r="C89" s="18" t="n">
         <v>46225</v>
       </c>
       <c r="D89" s="10" t="n">
@@ -2936,7 +3534,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C90" s="9" t="n">
+      <c r="C90" s="18" t="n">
         <v>46225</v>
       </c>
       <c r="D90" s="10" t="n">
@@ -2963,7 +3561,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C91" s="9" t="n">
+      <c r="C91" s="18" t="n">
         <v>46225</v>
       </c>
       <c r="D91" s="10" t="n">
@@ -2990,7 +3588,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C92" s="9" t="n">
+      <c r="C92" s="18" t="n">
         <v>46225</v>
       </c>
       <c r="D92" s="10" t="n">
@@ -3017,7 +3615,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C93" s="9" t="n">
+      <c r="C93" s="18" t="n">
         <v>46226</v>
       </c>
       <c r="D93" s="10" t="n">
@@ -3048,7 +3646,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C94" s="9" t="n">
+      <c r="C94" s="18" t="n">
         <v>46226</v>
       </c>
       <c r="D94" s="10" t="n">
@@ -3075,7 +3673,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C95" s="9" t="n">
+      <c r="C95" s="18" t="n">
         <v>46226</v>
       </c>
       <c r="D95" s="10" t="n">
@@ -3102,7 +3700,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C96" s="9" t="n">
+      <c r="C96" s="18" t="n">
         <v>46226</v>
       </c>
       <c r="D96" s="10" t="n">
@@ -3129,7 +3727,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C97" s="9" t="n">
+      <c r="C97" s="18" t="n">
         <v>46226</v>
       </c>
       <c r="D97" s="10" t="n">
@@ -3156,7 +3754,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C98" s="9" t="n">
+      <c r="C98" s="18" t="n">
         <v>46226</v>
       </c>
       <c r="D98" s="10" t="n">
@@ -3183,7 +3781,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C99" s="9" t="n">
+      <c r="C99" s="18" t="n">
         <v>46227</v>
       </c>
       <c r="D99" s="10" t="n">
@@ -3218,7 +3816,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C100" s="9" t="n">
+      <c r="C100" s="18" t="n">
         <v>46227</v>
       </c>
       <c r="D100" s="10" t="n">
@@ -3249,7 +3847,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C101" s="9" t="n">
+      <c r="C101" s="18" t="n">
         <v>46227</v>
       </c>
       <c r="D101" s="10" t="n">
@@ -3276,7 +3874,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C102" s="9" t="n">
+      <c r="C102" s="18" t="n">
         <v>46227</v>
       </c>
       <c r="D102" s="10" t="n">
@@ -3303,7 +3901,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C103" s="9" t="n">
+      <c r="C103" s="18" t="n">
         <v>46227</v>
       </c>
       <c r="D103" s="10" t="n">
@@ -3330,7 +3928,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C104" s="9" t="n">
+      <c r="C104" s="18" t="n">
         <v>46228</v>
       </c>
       <c r="D104" s="10" t="n">
@@ -3357,7 +3955,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C105" s="9" t="n">
+      <c r="C105" s="18" t="n">
         <v>46228</v>
       </c>
       <c r="D105" s="10" t="n">
@@ -3384,7 +3982,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C106" s="9" t="n">
+      <c r="C106" s="18" t="n">
         <v>46229</v>
       </c>
       <c r="D106" s="10" t="n">
@@ -3411,7 +4009,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C107" s="9" t="n">
+      <c r="C107" s="18" t="n">
         <v>46230</v>
       </c>
       <c r="D107" s="10" t="n">
@@ -3446,7 +4044,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C108" s="9" t="n">
+      <c r="C108" s="18" t="n">
         <v>46230</v>
       </c>
       <c r="D108" s="10" t="n">
@@ -3477,7 +4075,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C109" s="9" t="n">
+      <c r="C109" s="18" t="n">
         <v>46230</v>
       </c>
       <c r="D109" s="10" t="n">
@@ -3504,7 +4102,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C110" s="9" t="n">
+      <c r="C110" s="18" t="n">
         <v>46230</v>
       </c>
       <c r="D110" s="10" t="n">
@@ -3531,7 +4129,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C111" s="9" t="n">
+      <c r="C111" s="18" t="n">
         <v>46230</v>
       </c>
       <c r="D111" s="10" t="n">
@@ -3558,7 +4156,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C112" s="9" t="n">
+      <c r="C112" s="18" t="n">
         <v>46231</v>
       </c>
       <c r="D112" s="10" t="n">
@@ -3589,7 +4187,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C113" s="9" t="n">
+      <c r="C113" s="18" t="n">
         <v>46231</v>
       </c>
       <c r="D113" s="10" t="n">
@@ -3616,7 +4214,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C114" s="9" t="n">
+      <c r="C114" s="18" t="n">
         <v>46231</v>
       </c>
       <c r="D114" s="10" t="n">
@@ -3643,7 +4241,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C115" s="9" t="n">
+      <c r="C115" s="18" t="n">
         <v>46231</v>
       </c>
       <c r="D115" s="10" t="n">
@@ -3670,7 +4268,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C116" s="9" t="n">
+      <c r="C116" s="18" t="n">
         <v>46231</v>
       </c>
       <c r="D116" s="10" t="n">
@@ -3697,7 +4295,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C117" s="9" t="n">
+      <c r="C117" s="18" t="n">
         <v>46232</v>
       </c>
       <c r="D117" s="10" t="n">
@@ -3732,7 +4330,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C118" s="9" t="n">
+      <c r="C118" s="18" t="n">
         <v>46232</v>
       </c>
       <c r="D118" s="10" t="n">
@@ -3763,7 +4361,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C119" s="9" t="n">
+      <c r="C119" s="18" t="n">
         <v>46232</v>
       </c>
       <c r="D119" s="10" t="n">
@@ -3790,7 +4388,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C120" s="9" t="n">
+      <c r="C120" s="18" t="n">
         <v>46232</v>
       </c>
       <c r="D120" s="10" t="n">
@@ -3817,7 +4415,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C121" s="9" t="n">
+      <c r="C121" s="18" t="n">
         <v>46232</v>
       </c>
       <c r="D121" s="10" t="n">
@@ -3844,7 +4442,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C122" s="9" t="n">
+      <c r="C122" s="18" t="n">
         <v>46233</v>
       </c>
       <c r="D122" s="10" t="n">
@@ -3875,7 +4473,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C123" s="9" t="n">
+      <c r="C123" s="18" t="n">
         <v>46233</v>
       </c>
       <c r="D123" s="10" t="n">
@@ -3902,7 +4500,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C124" s="9" t="n">
+      <c r="C124" s="18" t="n">
         <v>46233</v>
       </c>
       <c r="D124" s="10" t="n">
@@ -3929,7 +4527,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C125" s="9" t="n">
+      <c r="C125" s="18" t="n">
         <v>46233</v>
       </c>
       <c r="D125" s="10" t="n">
@@ -3956,7 +4554,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C126" s="9" t="n">
+      <c r="C126" s="18" t="n">
         <v>46233</v>
       </c>
       <c r="D126" s="10" t="n">
@@ -3983,7 +4581,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C127" s="9" t="n">
+      <c r="C127" s="18" t="n">
         <v>46234</v>
       </c>
       <c r="D127" s="10" t="n">
@@ -4018,7 +4616,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C128" s="9" t="n">
+      <c r="C128" s="18" t="n">
         <v>46234</v>
       </c>
       <c r="D128" s="10" t="n">
@@ -4049,7 +4647,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C129" s="9" t="n">
+      <c r="C129" s="18" t="n">
         <v>46234</v>
       </c>
       <c r="D129" s="10" t="n">
@@ -4076,7 +4674,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C130" s="9" t="n">
+      <c r="C130" s="18" t="n">
         <v>46234</v>
       </c>
       <c r="D130" s="10" t="n">
@@ -4103,7 +4701,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C131" s="9" t="n">
+      <c r="C131" s="18" t="n">
         <v>46234</v>
       </c>
       <c r="D131" s="10" t="n">
@@ -4130,7 +4728,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C132" s="9" t="n">
+      <c r="C132" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D132" s="10" t="n">
@@ -4165,7 +4763,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C133" s="9" t="n">
+      <c r="C133" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D133" s="10" t="n">
@@ -4196,7 +4794,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C134" s="9" t="n">
+      <c r="C134" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D134" s="10" t="n">
@@ -4223,7 +4821,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C135" s="9" t="n">
+      <c r="C135" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D135" s="10" t="n">
@@ -4250,7 +4848,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C136" s="9" t="n">
+      <c r="C136" s="18" t="n">
         <v>46220</v>
       </c>
       <c r="D136" s="10" t="n">
@@ -4277,7 +4875,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C137" s="9" t="n"/>
+      <c r="C137" s="18" t="n"/>
       <c r="D137" s="10" t="n"/>
       <c r="E137" s="11" t="n"/>
       <c r="F137" s="11" t="n"/>
@@ -4290,7 +4888,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C138" s="9" t="n"/>
+      <c r="C138" s="18" t="n"/>
       <c r="D138" s="10" t="n"/>
       <c r="E138" s="11" t="n"/>
       <c r="F138" s="11" t="n"/>
@@ -4303,7 +4901,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C139" s="9" t="n"/>
+      <c r="C139" s="18" t="n"/>
       <c r="D139" s="10" t="n"/>
       <c r="E139" s="11" t="n"/>
       <c r="F139" s="11" t="n"/>
@@ -4316,7 +4914,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C140" s="9" t="n"/>
+      <c r="C140" s="18" t="n"/>
       <c r="D140" s="10" t="n"/>
       <c r="E140" s="11" t="n"/>
       <c r="F140" s="11" t="n"/>
@@ -4329,7 +4927,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C141" s="9" t="n"/>
+      <c r="C141" s="18" t="n"/>
       <c r="D141" s="10" t="n"/>
       <c r="E141" s="11" t="n"/>
       <c r="F141" s="11" t="n"/>
@@ -4342,7 +4940,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C142" s="9" t="n"/>
+      <c r="C142" s="18" t="n"/>
       <c r="D142" s="10" t="n"/>
       <c r="E142" s="11" t="n"/>
       <c r="F142" s="11" t="n"/>
@@ -4355,7 +4953,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C143" s="9" t="n"/>
+      <c r="C143" s="18" t="n"/>
       <c r="D143" s="10" t="n"/>
       <c r="E143" s="11" t="n"/>
       <c r="F143" s="11" t="n"/>
@@ -4368,7 +4966,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C144" s="9" t="n"/>
+      <c r="C144" s="18" t="n"/>
       <c r="D144" s="10" t="n"/>
       <c r="E144" s="11" t="n"/>
       <c r="F144" s="11" t="n"/>
@@ -4381,7 +4979,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C145" s="9" t="n"/>
+      <c r="C145" s="18" t="n"/>
       <c r="D145" s="10" t="n"/>
       <c r="E145" s="11" t="n"/>
       <c r="F145" s="11" t="n"/>
@@ -4394,7 +4992,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C146" s="9" t="n"/>
+      <c r="C146" s="18" t="n"/>
       <c r="D146" s="10" t="n"/>
       <c r="E146" s="11" t="n"/>
       <c r="F146" s="11" t="n"/>
@@ -4407,7 +5005,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C147" s="9" t="n"/>
+      <c r="C147" s="18" t="n"/>
       <c r="D147" s="10" t="n"/>
       <c r="E147" s="11" t="n"/>
       <c r="F147" s="11" t="n"/>
@@ -4420,7 +5018,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C148" s="9" t="n"/>
+      <c r="C148" s="18" t="n"/>
       <c r="D148" s="10" t="n"/>
       <c r="E148" s="11" t="n"/>
       <c r="F148" s="11" t="n"/>
@@ -4433,7 +5031,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C149" s="9" t="n"/>
+      <c r="C149" s="18" t="n"/>
       <c r="D149" s="10" t="n"/>
       <c r="E149" s="11" t="n"/>
       <c r="F149" s="11" t="n"/>
@@ -4446,7 +5044,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C150" s="9" t="n"/>
+      <c r="C150" s="18" t="n"/>
       <c r="D150" s="10" t="n"/>
       <c r="E150" s="11" t="n"/>
       <c r="F150" s="11" t="n"/>
@@ -4459,7 +5057,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C151" s="9" t="n"/>
+      <c r="C151" s="18" t="n"/>
       <c r="D151" s="10" t="n"/>
       <c r="E151" s="11" t="n"/>
       <c r="F151" s="11" t="n"/>
@@ -4472,7 +5070,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C152" s="9" t="n"/>
+      <c r="C152" s="18" t="n"/>
       <c r="D152" s="10" t="n"/>
       <c r="E152" s="11" t="n"/>
       <c r="F152" s="11" t="n"/>
@@ -4485,7 +5083,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C153" s="9" t="n"/>
+      <c r="C153" s="18" t="n"/>
       <c r="D153" s="10" t="n"/>
       <c r="E153" s="11" t="n"/>
       <c r="F153" s="11" t="n"/>
@@ -4498,7 +5096,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C154" s="9" t="n"/>
+      <c r="C154" s="18" t="n"/>
       <c r="D154" s="10" t="n"/>
       <c r="E154" s="11" t="n"/>
       <c r="F154" s="11" t="n"/>
@@ -4511,7 +5109,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C155" s="9" t="n"/>
+      <c r="C155" s="18" t="n"/>
       <c r="D155" s="10" t="n"/>
       <c r="E155" s="11" t="n"/>
       <c r="F155" s="11" t="n"/>
@@ -4524,7 +5122,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C156" s="9" t="n"/>
+      <c r="C156" s="18" t="n"/>
       <c r="D156" s="10" t="n"/>
       <c r="E156" s="11" t="n"/>
       <c r="F156" s="11" t="n"/>
@@ -4537,7 +5135,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C157" s="9" t="n"/>
+      <c r="C157" s="18" t="n"/>
       <c r="D157" s="10" t="n"/>
       <c r="E157" s="11" t="n"/>
       <c r="F157" s="11" t="n"/>
@@ -4550,7 +5148,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C158" s="9" t="n"/>
+      <c r="C158" s="18" t="n"/>
       <c r="D158" s="10" t="n"/>
       <c r="E158" s="11" t="n"/>
       <c r="F158" s="11" t="n"/>
@@ -4563,7 +5161,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C159" s="9" t="n"/>
+      <c r="C159" s="18" t="n"/>
       <c r="D159" s="10" t="n"/>
       <c r="E159" s="11" t="n"/>
       <c r="F159" s="11" t="n"/>
@@ -4576,7 +5174,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C160" s="9" t="n"/>
+      <c r="C160" s="18" t="n"/>
       <c r="D160" s="10" t="n"/>
       <c r="E160" s="11" t="n"/>
       <c r="F160" s="11" t="n"/>
@@ -4589,7 +5187,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C161" s="9" t="n"/>
+      <c r="C161" s="18" t="n"/>
       <c r="D161" s="10" t="n"/>
       <c r="E161" s="11" t="n"/>
       <c r="F161" s="11" t="n"/>
@@ -4602,7 +5200,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C162" s="9" t="n"/>
+      <c r="C162" s="18" t="n"/>
       <c r="D162" s="10" t="n"/>
       <c r="E162" s="11" t="n"/>
       <c r="F162" s="11" t="n"/>
@@ -4615,7 +5213,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C163" s="9" t="n"/>
+      <c r="C163" s="18" t="n"/>
       <c r="D163" s="10" t="n"/>
       <c r="E163" s="11" t="n"/>
       <c r="F163" s="11" t="n"/>
@@ -4628,7 +5226,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C164" s="9" t="n"/>
+      <c r="C164" s="18" t="n"/>
       <c r="D164" s="10" t="n"/>
       <c r="E164" s="11" t="n"/>
       <c r="F164" s="11" t="n"/>
@@ -4641,7 +5239,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C165" s="9" t="n"/>
+      <c r="C165" s="18" t="n"/>
       <c r="D165" s="10" t="n"/>
       <c r="E165" s="11" t="n"/>
       <c r="F165" s="11" t="n"/>
@@ -4654,7 +5252,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C166" s="9" t="n"/>
+      <c r="C166" s="18" t="n"/>
       <c r="D166" s="10" t="n"/>
       <c r="E166" s="11" t="n"/>
       <c r="F166" s="11" t="n"/>
@@ -4667,7 +5265,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C167" s="9" t="n"/>
+      <c r="C167" s="18" t="n"/>
       <c r="D167" s="10" t="n"/>
       <c r="E167" s="11" t="n"/>
       <c r="F167" s="11" t="n"/>
@@ -4680,7 +5278,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C168" s="9" t="n"/>
+      <c r="C168" s="18" t="n"/>
       <c r="D168" s="10" t="n"/>
       <c r="E168" s="11" t="n"/>
       <c r="F168" s="11" t="n"/>
@@ -4693,7 +5291,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C169" s="9" t="n"/>
+      <c r="C169" s="18" t="n"/>
       <c r="D169" s="10" t="n"/>
       <c r="E169" s="11" t="n"/>
       <c r="F169" s="11" t="n"/>
@@ -4706,7 +5304,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C170" s="9" t="n"/>
+      <c r="C170" s="18" t="n"/>
       <c r="D170" s="10" t="n"/>
       <c r="E170" s="11" t="n"/>
       <c r="F170" s="11" t="n"/>
@@ -4719,7 +5317,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C171" s="9" t="n"/>
+      <c r="C171" s="18" t="n"/>
       <c r="D171" s="10" t="n"/>
       <c r="E171" s="11" t="n"/>
       <c r="F171" s="11" t="n"/>
@@ -4732,7 +5330,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C172" s="9" t="n"/>
+      <c r="C172" s="18" t="n"/>
       <c r="D172" s="10" t="n"/>
       <c r="E172" s="11" t="n"/>
       <c r="F172" s="11" t="n"/>
@@ -4745,7 +5343,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C173" s="9" t="n"/>
+      <c r="C173" s="18" t="n"/>
       <c r="D173" s="10" t="n"/>
       <c r="E173" s="11" t="n"/>
       <c r="F173" s="11" t="n"/>
@@ -4758,7 +5356,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C174" s="9" t="n"/>
+      <c r="C174" s="18" t="n"/>
       <c r="D174" s="10" t="n"/>
       <c r="E174" s="11" t="n"/>
       <c r="F174" s="11" t="n"/>
@@ -4771,7 +5369,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C175" s="9" t="n"/>
+      <c r="C175" s="18" t="n"/>
       <c r="D175" s="10" t="n"/>
       <c r="E175" s="11" t="n"/>
       <c r="F175" s="11" t="n"/>
@@ -4784,7 +5382,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C176" s="9" t="n"/>
+      <c r="C176" s="18" t="n"/>
       <c r="D176" s="10" t="n"/>
       <c r="E176" s="11" t="n"/>
       <c r="F176" s="11" t="n"/>
@@ -4797,7 +5395,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C177" s="9" t="n"/>
+      <c r="C177" s="18" t="n"/>
       <c r="D177" s="10" t="n"/>
       <c r="E177" s="11" t="n"/>
       <c r="F177" s="11" t="n"/>
@@ -4810,7 +5408,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C178" s="9" t="n"/>
+      <c r="C178" s="18" t="n"/>
       <c r="D178" s="10" t="n"/>
       <c r="E178" s="11" t="n"/>
       <c r="F178" s="11" t="n"/>
@@ -4823,7 +5421,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C179" s="9" t="n"/>
+      <c r="C179" s="18" t="n"/>
       <c r="D179" s="10" t="n"/>
       <c r="E179" s="11" t="n"/>
       <c r="F179" s="11" t="n"/>
@@ -4836,7 +5434,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C180" s="9" t="n"/>
+      <c r="C180" s="18" t="n"/>
       <c r="D180" s="10" t="n"/>
       <c r="E180" s="11" t="n"/>
       <c r="F180" s="11" t="n"/>
@@ -4849,7 +5447,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C181" s="9" t="n"/>
+      <c r="C181" s="18" t="n"/>
       <c r="D181" s="10" t="n"/>
       <c r="E181" s="11" t="n"/>
       <c r="F181" s="11" t="n"/>
@@ -4862,7 +5460,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C182" s="9" t="n"/>
+      <c r="C182" s="18" t="n"/>
       <c r="D182" s="10" t="n"/>
       <c r="E182" s="11" t="n"/>
       <c r="F182" s="11" t="n"/>
@@ -4875,7 +5473,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C183" s="9" t="n"/>
+      <c r="C183" s="18" t="n"/>
       <c r="D183" s="10" t="n"/>
       <c r="E183" s="11" t="n"/>
       <c r="F183" s="11" t="n"/>
@@ -4888,7 +5486,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C184" s="9" t="n"/>
+      <c r="C184" s="18" t="n"/>
       <c r="D184" s="10" t="n"/>
       <c r="E184" s="11" t="n"/>
       <c r="F184" s="11" t="n"/>
@@ -4901,7 +5499,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C185" s="9" t="n"/>
+      <c r="C185" s="18" t="n"/>
       <c r="D185" s="10" t="n"/>
       <c r="E185" s="11" t="n"/>
       <c r="F185" s="11" t="n"/>
@@ -4914,7 +5512,7 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C186" s="9" t="n"/>
+      <c r="C186" s="18" t="n"/>
       <c r="D186" s="10" t="n"/>
       <c r="E186" s="11" t="n"/>
       <c r="F186" s="11" t="n"/>
@@ -4923,9 +5521,16 @@
       <c r="I186" s="12" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="9">
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="B2:I2"/>
     <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="K5:N5"/>
   </mergeCells>
   <dataValidations count="7">
     <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>

<commit_message>
Add redesigned Daily Rollup tab; fix duplicated day-of-strategy rows
Step 4 of the Call Delivery streamlining roadmap:

- Daily Rollup tab in the master workbook: pick a Strategy Date (or
  =TODAY()) and the morning sheet assembles itself from the Consolidated
  table via a hidden key/lookup helper - hourly grid per group with
  color-coded pass types (AMs/Branch/WFO/Blitz/TSC/Vendor), pass counts,
  special instructions, coverage and hours-of-operation sections.
- Parser fix: the old workbook's hidden row-97 lookup row duplicated the
  current day's passes on every group sheet; intake generation now reads
  only the calendar block (628 unique passes, was 655 with duplicates).
- Times render in the familiar 8:30a / 1:30p style.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DBbqxUN9AD2FdtJjEWSJGT
</commit_message>
<xml_diff>
--- a/call-delivery/intake/2026-07/Auto.xlsx
+++ b/call-delivery/intake/2026-07/Auto.xlsx
@@ -272,8 +272,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblSchedule" displayName="tblSchedule" ref="B9:I186" headerRowCount="1">
-  <autoFilter ref="B9:I186"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblSchedule" displayName="tblSchedule" ref="B9:I181" headerRowCount="1">
+  <autoFilter ref="B9:I181"/>
   <tableColumns count="8">
     <tableColumn id="2" name="Business Group"/>
     <tableColumn id="3" name="Date"/>
@@ -578,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N186"/>
+  <dimension ref="B2:N181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -4728,65 +4728,25 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C132" s="18" t="n">
-        <v>46220</v>
-      </c>
-      <c r="D132" s="10" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="E132" s="11" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="F132" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G132" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H132" s="11" t="inlineStr">
-        <is>
-          <t>AMs</t>
-        </is>
-      </c>
-      <c r="I132" s="12" t="inlineStr">
-        <is>
-          <t>Slowpay AM Daily</t>
-        </is>
-      </c>
+      <c r="C132" s="18" t="n"/>
+      <c r="D132" s="10" t="n"/>
+      <c r="E132" s="11" t="n"/>
+      <c r="F132" s="11" t="n"/>
+      <c r="G132" s="11" t="n"/>
+      <c r="H132" s="11" t="n"/>
+      <c r="I132" s="12" t="n"/>
     </row>
     <row r="133">
       <c r="B133" s="8">
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C133" s="18" t="n">
-        <v>46220</v>
-      </c>
-      <c r="D133" s="10" t="n">
-        <v>0.4791666666666667</v>
-      </c>
-      <c r="E133" s="11" t="inlineStr">
-        <is>
-          <t>C-M-P</t>
-        </is>
-      </c>
-      <c r="F133" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G133" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H133" s="11" t="inlineStr">
-        <is>
-          <t>AMs</t>
-        </is>
-      </c>
+      <c r="C133" s="18" t="n"/>
+      <c r="D133" s="10" t="n"/>
+      <c r="E133" s="11" t="n"/>
+      <c r="F133" s="11" t="n"/>
+      <c r="G133" s="11" t="n"/>
+      <c r="H133" s="11" t="n"/>
       <c r="I133" s="12" t="n"/>
     </row>
     <row r="134">
@@ -4794,26 +4754,12 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C134" s="18" t="n">
-        <v>46220</v>
-      </c>
-      <c r="D134" s="10" t="n">
-        <v>0.5625</v>
-      </c>
+      <c r="C134" s="18" t="n"/>
+      <c r="D134" s="10" t="n"/>
       <c r="E134" s="11" t="n"/>
-      <c r="F134" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G134" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="H134" s="11" t="inlineStr">
-        <is>
-          <t>WFO</t>
-        </is>
-      </c>
+      <c r="F134" s="11" t="n"/>
+      <c r="G134" s="11" t="n"/>
+      <c r="H134" s="11" t="n"/>
       <c r="I134" s="12" t="n"/>
     </row>
     <row r="135">
@@ -4821,26 +4767,12 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C135" s="18" t="n">
-        <v>46220</v>
-      </c>
-      <c r="D135" s="10" t="n">
-        <v>0.7083333333333334</v>
-      </c>
+      <c r="C135" s="18" t="n"/>
+      <c r="D135" s="10" t="n"/>
       <c r="E135" s="11" t="n"/>
-      <c r="F135" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G135" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="H135" s="11" t="inlineStr">
-        <is>
-          <t>Blitz</t>
-        </is>
-      </c>
+      <c r="F135" s="11" t="n"/>
+      <c r="G135" s="11" t="n"/>
+      <c r="H135" s="11" t="n"/>
       <c r="I135" s="12" t="n"/>
     </row>
     <row r="136">
@@ -4848,26 +4780,12 @@
         <f>IF($C$5="","",$C$5)</f>
         <v/>
       </c>
-      <c r="C136" s="18" t="n">
-        <v>46220</v>
-      </c>
-      <c r="D136" s="10" t="n">
-        <v>0.8333333333333334</v>
-      </c>
+      <c r="C136" s="18" t="n"/>
+      <c r="D136" s="10" t="n"/>
       <c r="E136" s="11" t="n"/>
-      <c r="F136" s="11" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G136" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="H136" s="11" t="inlineStr">
-        <is>
-          <t>TSC (All)</t>
-        </is>
-      </c>
+      <c r="F136" s="11" t="n"/>
+      <c r="G136" s="11" t="n"/>
+      <c r="H136" s="11" t="n"/>
       <c r="I136" s="12" t="n"/>
     </row>
     <row r="137">
@@ -5454,71 +5372,6 @@
       <c r="G181" s="11" t="n"/>
       <c r="H181" s="11" t="n"/>
       <c r="I181" s="12" t="n"/>
-    </row>
-    <row r="182">
-      <c r="B182" s="8">
-        <f>IF($C$5="","",$C$5)</f>
-        <v/>
-      </c>
-      <c r="C182" s="18" t="n"/>
-      <c r="D182" s="10" t="n"/>
-      <c r="E182" s="11" t="n"/>
-      <c r="F182" s="11" t="n"/>
-      <c r="G182" s="11" t="n"/>
-      <c r="H182" s="11" t="n"/>
-      <c r="I182" s="12" t="n"/>
-    </row>
-    <row r="183">
-      <c r="B183" s="8">
-        <f>IF($C$5="","",$C$5)</f>
-        <v/>
-      </c>
-      <c r="C183" s="18" t="n"/>
-      <c r="D183" s="10" t="n"/>
-      <c r="E183" s="11" t="n"/>
-      <c r="F183" s="11" t="n"/>
-      <c r="G183" s="11" t="n"/>
-      <c r="H183" s="11" t="n"/>
-      <c r="I183" s="12" t="n"/>
-    </row>
-    <row r="184">
-      <c r="B184" s="8">
-        <f>IF($C$5="","",$C$5)</f>
-        <v/>
-      </c>
-      <c r="C184" s="18" t="n"/>
-      <c r="D184" s="10" t="n"/>
-      <c r="E184" s="11" t="n"/>
-      <c r="F184" s="11" t="n"/>
-      <c r="G184" s="11" t="n"/>
-      <c r="H184" s="11" t="n"/>
-      <c r="I184" s="12" t="n"/>
-    </row>
-    <row r="185">
-      <c r="B185" s="8">
-        <f>IF($C$5="","",$C$5)</f>
-        <v/>
-      </c>
-      <c r="C185" s="18" t="n"/>
-      <c r="D185" s="10" t="n"/>
-      <c r="E185" s="11" t="n"/>
-      <c r="F185" s="11" t="n"/>
-      <c r="G185" s="11" t="n"/>
-      <c r="H185" s="11" t="n"/>
-      <c r="I185" s="12" t="n"/>
-    </row>
-    <row r="186">
-      <c r="B186" s="8">
-        <f>IF($C$5="","",$C$5)</f>
-        <v/>
-      </c>
-      <c r="C186" s="18" t="n"/>
-      <c r="D186" s="10" t="n"/>
-      <c r="E186" s="11" t="n"/>
-      <c r="F186" s="11" t="n"/>
-      <c r="G186" s="11" t="n"/>
-      <c r="H186" s="11" t="n"/>
-      <c r="I186" s="12" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -5536,23 +5389,23 @@
     <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Lists!$A$2:$A$21</formula1>
     </dataValidation>
-    <dataValidation sqref="E10:E186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E10:E181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Lists!$B$2:$B$12</formula1>
     </dataValidation>
-    <dataValidation sqref="F10:F186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F10:F181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Lists!$D$2:$D$31</formula1>
     </dataValidation>
-    <dataValidation sqref="H10:H186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H10:H181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Lists!$C$2:$C$15</formula1>
     </dataValidation>
-    <dataValidation sqref="G10:G186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="G10:G181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="C10:C186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThanOrEqual">
+    <dataValidation sqref="C10:C181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThanOrEqual">
       <formula1>DATE(2020,1,1)</formula1>
     </dataValidation>
-    <dataValidation sqref="D10:D186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="time" operator="between">
+    <dataValidation sqref="D10:D181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="time" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>

</xml_diff>